<commit_message>
MO-630: add missing keys
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/07-accepted-prn.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/07-accepted-prn.xlsx
@@ -76,7 +76,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1" hidden="1"/>
@@ -273,8 +273,50 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_recyclingNoteStatus.en.resx::reprocessing_site</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_recyclingNoteStatus.en.resx</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reprocessing_site</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-accepted-single</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/accepted-prn/{id}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reprocessing site</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Safle ailbrosesu</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H8"/>
+  <autoFilter ref="A5:H9"/>
   <mergeCells count="3">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="F2:H2"/>

</xml_diff>

<commit_message>
MO-575: add welsh copy for 2025
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/07-accepted-prn.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/07-accepted-prn.xlsx
@@ -180,7 +180,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Derbynioch chi y {0} yma at eich rhwymedigaethau ailgylchu {1}</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -222,7 +222,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Rydych chi wedi cyfrannu {0} o dunelli at eich rhwymedigaeth ailgylchu ar gyfer {1}.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">

</xml_diff>

<commit_message>
MO-575: add welsh copy for 2025 (#379)
* MO-575: add welsh copy for 2025

* fix unit tests
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/07-accepted-prn.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/07-accepted-prn.xlsx
@@ -180,7 +180,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Derbynioch chi y {0} yma at eich rhwymedigaethau ailgylchu {1}</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -222,7 +222,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Rydych chi wedi cyfrannu {0} o dunelli at eich rhwymedigaeth ailgylchu ar gyfer {1}.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">

</xml_diff>